<commit_message>
updated Attack Surface Analysis - Analysis Procedure (images / license) and associated issue template (legend) annotation)
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/templates/AVCDL attack surface analysis issues template.xlsx
+++ b/distribution/reference_documents/templates/AVCDL attack surface analysis issues template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D47459-AF53-A343-B817-33A378DA14C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C29D06A6-3A53-104E-A6B1-8C8DEF2E90E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="41880" yWindow="1360" windowWidth="30240" windowHeight="18880" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
@@ -203,7 +203,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -287,6 +287,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FF0070C0"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -348,7 +355,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -406,6 +413,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="45"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1392,7 +1400,7 @@
       <c r="A6" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="29" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="21"/>
@@ -1402,7 +1410,7 @@
       <c r="A7" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="29" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="21"/>

</xml_diff>